<commit_message>
Previsão de faturamento: mensal do ano 1, anual 12 anos e formulário oficial de Receitas
- previsao-faturamento.xlsx: Linha do Tempo (implantação ago-dez/2026 + 12 meses de
  operação), Mensal Ano 1 por produto (R$ 35,6 mil em jan a R$ 366 mil em out;
  total R$ 2.750.000), Anual 12 anos, Sazonalidade fundamentada e Conferência
- receitas-bnb.xlsx: layout oficial da aba Receitas/Atividades (Qtd. Atual = 0;
  Qtd. Projetada = regime; % de Utilização ano 1 de 43-72% conforme produto)
- previsao-faturamento.md: método em 3 camadas (mix por absorção, entrada escalonada
  por produto, sazonalidade ABCP/CBIC) + alerta do teto EPP em valores nominais
- Ano 1 usa 103 de 210 dias efetivos; nenhum mês acima de 76% da capacidade mensal
- Referência cruzada na memória BNB e no kit de defesa

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CKyLR5v4criVdVXwyZSi7P
</commit_message>
<xml_diff>
--- a/estudo-mercado-gtk/dossie-bnb/memoria-calculo-bnb.xlsx
+++ b/estudo-mercado-gtk/dossie-bnb/memoria-calculo-bnb.xlsx
@@ -783,15 +783,15 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C15:E15"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C15:E15"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="C10:E10"/>
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1106,6 +1106,13 @@
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Receita do regime derivada do mix (não afirmada): Σ volume × preço = R$ 4.790.992 ≈ 4.791.000. Detalhe na aba G31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Abertura mensal do ano 1 e formulário oficial de Receitas/Atividades: ver previsao-faturamento.xlsx e receitas-bnb.xlsx (mesma pasta).</t>
         </is>
       </c>
     </row>

</xml_diff>